<commit_message>
captured screenshot of failed tests using Listners
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shraddha\Intellej_workspace\TestAutoFramework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49AA74FD-9867-4D0B-96DA-E14322897086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF0E624-AF8E-4E75-BA71-C00CC8F195A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{99E50069-335D-4957-B737-0BFDEE988E12}"/>
   </bookViews>
@@ -30,13 +30,13 @@
     <t>unmeshtemkar@zohomail.in</t>
   </si>
   <si>
-    <t>1995@umaaa</t>
-  </si>
-  <si>
     <t>kalaskarshraddha.777@gmail.com</t>
   </si>
   <si>
     <t>Veer@Shrad@1008</t>
+  </si>
+  <si>
+    <t>1995@umaaa</t>
   </si>
 </sst>
 </file>
@@ -411,15 +411,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>